<commit_message>
Polish Chinese copy for finance narrative modules
</commit_message>
<xml_diff>
--- a/public/sample-data/enterprise-finance-sample.xlsx
+++ b/public/sample-data/enterprise-finance-sample.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12375" activeTab="5"/>
+    <workbookView windowWidth="28800" windowHeight="12375" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard_Notes" sheetId="1" r:id="rId1"/>
@@ -2889,6 +2889,18 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GLActualsTable" displayName="GLActualsTable" ref="A1:O301">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:O301" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="6100"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="13">
+      <filters>
+        <filter val="CC300 Ops"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="15">
     <tableColumn id="1" name="Period"/>
     <tableColumn id="2" name="Entity"/>
@@ -15795,7 +15807,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" hidden="1" spans="1:26">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -15842,7 +15854,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:26">
+    <row r="3" hidden="1" spans="1:26">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -15889,7 +15901,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:26">
+    <row r="4" hidden="1" spans="1:26">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -15918,16 +15930,16 @@
         <v>22</v>
       </c>
       <c r="J4">
-        <v>-42188</v>
+        <v>-65747</v>
       </c>
       <c r="K4">
         <v>-43779</v>
       </c>
       <c r="L4">
-        <v>-43370</v>
+        <v>-53475</v>
       </c>
       <c r="M4">
-        <v>-40921</v>
+        <v>-35643</v>
       </c>
       <c r="N4" t="s">
         <v>76</v>
@@ -15965,7 +15977,7 @@
         <v>23</v>
       </c>
       <c r="J5">
-        <v>-13681</v>
+        <v>-34523</v>
       </c>
       <c r="K5">
         <v>-15294</v>
@@ -15974,7 +15986,7 @@
         <v>-14746</v>
       </c>
       <c r="M5">
-        <v>-13790</v>
+        <v>-24353</v>
       </c>
       <c r="N5" t="s">
         <v>84</v>
@@ -15983,7 +15995,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" hidden="1" spans="1:26">
       <c r="A6" t="s">
         <v>48</v>
       </c>
@@ -16030,7 +16042,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" hidden="1" spans="1:26">
       <c r="A7" t="s">
         <v>55</v>
       </c>
@@ -16077,7 +16089,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" hidden="1" spans="1:26">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -16124,7 +16136,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" hidden="1" spans="1:26">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -16171,7 +16183,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" hidden="1" spans="1:26">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -16218,7 +16230,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:26">
+    <row r="11" hidden="1" spans="1:26">
       <c r="A11" t="s">
         <v>49</v>
       </c>
@@ -16265,7 +16277,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" hidden="1" spans="1:26">
       <c r="A12" t="s">
         <v>48</v>
       </c>
@@ -16312,7 +16324,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" hidden="1" spans="1:26">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -16359,7 +16371,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" hidden="1" spans="1:26">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -16406,7 +16418,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" hidden="1" spans="1:26">
       <c r="A15" t="s">
         <v>54</v>
       </c>
@@ -16453,7 +16465,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:26">
+    <row r="16" hidden="1" spans="1:26">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -16500,7 +16512,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" hidden="1" spans="1:15">
       <c r="A17" t="s">
         <v>51</v>
       </c>
@@ -16547,7 +16559,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" hidden="1" spans="1:15">
       <c r="A18" t="s">
         <v>54</v>
       </c>
@@ -16594,7 +16606,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" hidden="1" spans="1:15">
       <c r="A19" t="s">
         <v>47</v>
       </c>
@@ -16641,7 +16653,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" hidden="1" spans="1:15">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -16688,7 +16700,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" hidden="1" spans="1:15">
       <c r="A21" t="s">
         <v>53</v>
       </c>
@@ -16735,7 +16747,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" hidden="1" spans="1:15">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -16782,7 +16794,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" hidden="1" spans="1:15">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -16829,7 +16841,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" hidden="1" spans="1:15">
       <c r="A24" t="s">
         <v>53</v>
       </c>
@@ -16876,7 +16888,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" hidden="1" spans="1:15">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -16923,7 +16935,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" hidden="1" spans="1:15">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -16970,7 +16982,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" hidden="1" spans="1:15">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -17017,7 +17029,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
+    <row r="28" hidden="1" spans="1:15">
       <c r="A28" t="s">
         <v>51</v>
       </c>
@@ -17064,7 +17076,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" hidden="1" spans="1:15">
       <c r="A29" t="s">
         <v>49</v>
       </c>
@@ -17111,7 +17123,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" hidden="1" spans="1:15">
       <c r="A30" t="s">
         <v>45</v>
       </c>
@@ -17158,7 +17170,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" hidden="1" spans="1:15">
       <c r="A31" t="s">
         <v>55</v>
       </c>
@@ -17205,7 +17217,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" hidden="1" spans="1:15">
       <c r="A32" t="s">
         <v>52</v>
       </c>
@@ -17252,7 +17264,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" hidden="1" spans="1:15">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -17299,7 +17311,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" hidden="1" spans="1:15">
       <c r="A34" t="s">
         <v>51</v>
       </c>
@@ -17346,7 +17358,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" hidden="1" spans="1:15">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -17393,7 +17405,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:15">
+    <row r="36" hidden="1" spans="1:15">
       <c r="A36" t="s">
         <v>55</v>
       </c>
@@ -17440,7 +17452,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" hidden="1" spans="1:15">
       <c r="A37" t="s">
         <v>50</v>
       </c>
@@ -17487,7 +17499,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" hidden="1" spans="1:15">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -17534,7 +17546,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:15">
+    <row r="39" hidden="1" spans="1:15">
       <c r="A39" t="s">
         <v>50</v>
       </c>
@@ -17581,7 +17593,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="40" spans="1:15">
+    <row r="40" hidden="1" spans="1:15">
       <c r="A40" t="s">
         <v>53</v>
       </c>
@@ -17628,7 +17640,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="41" spans="1:15">
+    <row r="41" hidden="1" spans="1:15">
       <c r="A41" t="s">
         <v>46</v>
       </c>
@@ -17675,7 +17687,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:15">
+    <row r="42" hidden="1" spans="1:15">
       <c r="A42" t="s">
         <v>51</v>
       </c>
@@ -17722,7 +17734,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="43" spans="1:15">
+    <row r="43" hidden="1" spans="1:15">
       <c r="A43" t="s">
         <v>53</v>
       </c>
@@ -17769,7 +17781,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:15">
+    <row r="44" hidden="1" spans="1:15">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -17816,7 +17828,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:15">
+    <row r="45" hidden="1" spans="1:15">
       <c r="A45" t="s">
         <v>52</v>
       </c>
@@ -17863,7 +17875,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="46" spans="1:15">
+    <row r="46" hidden="1" spans="1:15">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -17910,7 +17922,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="47" spans="1:15">
+    <row r="47" hidden="1" spans="1:15">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -17957,7 +17969,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="48" spans="1:15">
+    <row r="48" hidden="1" spans="1:15">
       <c r="A48" t="s">
         <v>45</v>
       </c>
@@ -18004,7 +18016,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="49" spans="1:15">
+    <row r="49" hidden="1" spans="1:15">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -18051,7 +18063,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="50" spans="1:15">
+    <row r="50" hidden="1" spans="1:15">
       <c r="A50" t="s">
         <v>49</v>
       </c>
@@ -18098,7 +18110,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="1:15">
+    <row r="51" hidden="1" spans="1:15">
       <c r="A51" t="s">
         <v>54</v>
       </c>
@@ -18145,7 +18157,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:15">
+    <row r="52" hidden="1" spans="1:15">
       <c r="A52" t="s">
         <v>52</v>
       </c>
@@ -18192,7 +18204,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="53" spans="1:15">
+    <row r="53" hidden="1" spans="1:15">
       <c r="A53" t="s">
         <v>51</v>
       </c>
@@ -18239,7 +18251,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="54" spans="1:15">
+    <row r="54" hidden="1" spans="1:15">
       <c r="A54" t="s">
         <v>52</v>
       </c>
@@ -18286,7 +18298,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="55" spans="1:15">
+    <row r="55" hidden="1" spans="1:15">
       <c r="A55" t="s">
         <v>50</v>
       </c>
@@ -18333,7 +18345,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="56" spans="1:15">
+    <row r="56" hidden="1" spans="1:15">
       <c r="A56" t="s">
         <v>48</v>
       </c>
@@ -18380,7 +18392,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="57" spans="1:15">
+    <row r="57" hidden="1" spans="1:15">
       <c r="A57" t="s">
         <v>52</v>
       </c>
@@ -18427,7 +18439,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
+    <row r="58" hidden="1" spans="1:15">
       <c r="A58" t="s">
         <v>53</v>
       </c>
@@ -18474,7 +18486,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="59" spans="1:15">
+    <row r="59" hidden="1" spans="1:15">
       <c r="A59" t="s">
         <v>48</v>
       </c>
@@ -18521,7 +18533,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="60" spans="1:15">
+    <row r="60" hidden="1" spans="1:15">
       <c r="A60" t="s">
         <v>50</v>
       </c>
@@ -18568,7 +18580,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="61" spans="1:15">
+    <row r="61" hidden="1" spans="1:15">
       <c r="A61" t="s">
         <v>55</v>
       </c>
@@ -18615,7 +18627,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="62" spans="1:15">
+    <row r="62" hidden="1" spans="1:15">
       <c r="A62" t="s">
         <v>53</v>
       </c>
@@ -18662,7 +18674,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="63" spans="1:15">
+    <row r="63" hidden="1" spans="1:15">
       <c r="A63" t="s">
         <v>54</v>
       </c>
@@ -18709,7 +18721,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="64" spans="1:15">
+    <row r="64" hidden="1" spans="1:15">
       <c r="A64" t="s">
         <v>47</v>
       </c>
@@ -18756,7 +18768,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="65" spans="1:15">
+    <row r="65" hidden="1" spans="1:15">
       <c r="A65" t="s">
         <v>36</v>
       </c>
@@ -18803,7 +18815,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="66" spans="1:15">
+    <row r="66" hidden="1" spans="1:15">
       <c r="A66" t="s">
         <v>45</v>
       </c>
@@ -18850,7 +18862,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="67" spans="1:15">
+    <row r="67" hidden="1" spans="1:15">
       <c r="A67" t="s">
         <v>47</v>
       </c>
@@ -18897,7 +18909,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:15">
+    <row r="68" hidden="1" spans="1:15">
       <c r="A68" t="s">
         <v>53</v>
       </c>
@@ -18944,7 +18956,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="69" spans="1:15">
+    <row r="69" hidden="1" spans="1:15">
       <c r="A69" t="s">
         <v>46</v>
       </c>
@@ -18991,7 +19003,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="70" spans="1:15">
+    <row r="70" hidden="1" spans="1:15">
       <c r="A70" t="s">
         <v>45</v>
       </c>
@@ -19038,7 +19050,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="71" spans="1:15">
+    <row r="71" hidden="1" spans="1:15">
       <c r="A71" t="s">
         <v>36</v>
       </c>
@@ -19085,7 +19097,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="72" spans="1:15">
+    <row r="72" hidden="1" spans="1:15">
       <c r="A72" t="s">
         <v>53</v>
       </c>
@@ -19132,7 +19144,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="73" spans="1:15">
+    <row r="73" hidden="1" spans="1:15">
       <c r="A73" t="s">
         <v>53</v>
       </c>
@@ -19179,7 +19191,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="74" spans="1:15">
+    <row r="74" hidden="1" spans="1:15">
       <c r="A74" t="s">
         <v>36</v>
       </c>
@@ -19226,7 +19238,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="75" spans="1:15">
+    <row r="75" hidden="1" spans="1:15">
       <c r="A75" t="s">
         <v>49</v>
       </c>
@@ -19273,7 +19285,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" spans="1:15">
+    <row r="76" hidden="1" spans="1:15">
       <c r="A76" t="s">
         <v>36</v>
       </c>
@@ -19320,7 +19332,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="77" spans="1:15">
+    <row r="77" hidden="1" spans="1:15">
       <c r="A77" t="s">
         <v>52</v>
       </c>
@@ -19414,7 +19426,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="79" spans="1:15">
+    <row r="79" hidden="1" spans="1:15">
       <c r="A79" t="s">
         <v>51</v>
       </c>
@@ -19461,7 +19473,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="80" spans="1:15">
+    <row r="80" hidden="1" spans="1:15">
       <c r="A80" t="s">
         <v>55</v>
       </c>
@@ -19555,7 +19567,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="82" spans="1:15">
+    <row r="82" hidden="1" spans="1:15">
       <c r="A82" t="s">
         <v>55</v>
       </c>
@@ -19602,7 +19614,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="83" spans="1:15">
+    <row r="83" hidden="1" spans="1:15">
       <c r="A83" t="s">
         <v>36</v>
       </c>
@@ -19649,7 +19661,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="84" spans="1:15">
+    <row r="84" hidden="1" spans="1:15">
       <c r="A84" t="s">
         <v>49</v>
       </c>
@@ -19696,7 +19708,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="85" spans="1:15">
+    <row r="85" hidden="1" spans="1:15">
       <c r="A85" t="s">
         <v>47</v>
       </c>
@@ -19743,7 +19755,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="86" spans="1:15">
+    <row r="86" hidden="1" spans="1:15">
       <c r="A86" t="s">
         <v>47</v>
       </c>
@@ -19790,7 +19802,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="87" spans="1:15">
+    <row r="87" hidden="1" spans="1:15">
       <c r="A87" t="s">
         <v>50</v>
       </c>
@@ -19837,7 +19849,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="88" spans="1:15">
+    <row r="88" hidden="1" spans="1:15">
       <c r="A88" t="s">
         <v>48</v>
       </c>
@@ -19884,7 +19896,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="89" spans="1:15">
+    <row r="89" hidden="1" spans="1:15">
       <c r="A89" t="s">
         <v>55</v>
       </c>
@@ -19931,7 +19943,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="90" spans="1:15">
+    <row r="90" hidden="1" spans="1:15">
       <c r="A90" t="s">
         <v>51</v>
       </c>
@@ -19978,7 +19990,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="91" spans="1:15">
+    <row r="91" hidden="1" spans="1:15">
       <c r="A91" t="s">
         <v>52</v>
       </c>
@@ -20025,7 +20037,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="92" spans="1:15">
+    <row r="92" hidden="1" spans="1:15">
       <c r="A92" t="s">
         <v>50</v>
       </c>
@@ -20072,7 +20084,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="93" spans="1:15">
+    <row r="93" hidden="1" spans="1:15">
       <c r="A93" t="s">
         <v>52</v>
       </c>
@@ -20119,7 +20131,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="94" spans="1:15">
+    <row r="94" hidden="1" spans="1:15">
       <c r="A94" t="s">
         <v>45</v>
       </c>
@@ -20166,7 +20178,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="95" spans="1:15">
+    <row r="95" hidden="1" spans="1:15">
       <c r="A95" t="s">
         <v>49</v>
       </c>
@@ -20213,7 +20225,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="96" spans="1:15">
+    <row r="96" hidden="1" spans="1:15">
       <c r="A96" t="s">
         <v>50</v>
       </c>
@@ -20260,7 +20272,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="97" spans="1:15">
+    <row r="97" hidden="1" spans="1:15">
       <c r="A97" t="s">
         <v>51</v>
       </c>
@@ -20286,19 +20298,19 @@
         <v>80</v>
       </c>
       <c r="I97" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J97">
-        <v>-32909</v>
+        <v>32909</v>
       </c>
       <c r="K97">
-        <v>-35502</v>
+        <v>35502</v>
       </c>
       <c r="L97">
-        <v>-32827</v>
+        <v>32827</v>
       </c>
       <c r="M97">
-        <v>-30460</v>
+        <v>30460</v>
       </c>
       <c r="N97" t="s">
         <v>92</v>
@@ -20307,7 +20319,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="98" spans="1:15">
+    <row r="98" hidden="1" spans="1:15">
       <c r="A98" t="s">
         <v>52</v>
       </c>
@@ -20354,7 +20366,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="99" spans="1:15">
+    <row r="99" hidden="1" spans="1:15">
       <c r="A99" t="s">
         <v>47</v>
       </c>
@@ -20401,7 +20413,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="100" spans="1:15">
+    <row r="100" hidden="1" spans="1:15">
       <c r="A100" t="s">
         <v>50</v>
       </c>
@@ -20448,7 +20460,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="101" spans="1:15">
+    <row r="101" hidden="1" spans="1:15">
       <c r="A101" t="s">
         <v>47</v>
       </c>
@@ -20495,7 +20507,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="102" spans="1:15">
+    <row r="102" hidden="1" spans="1:15">
       <c r="A102" t="s">
         <v>48</v>
       </c>
@@ -20542,7 +20554,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="103" spans="1:15">
+    <row r="103" hidden="1" spans="1:15">
       <c r="A103" t="s">
         <v>51</v>
       </c>
@@ -20589,7 +20601,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="104" spans="1:15">
+    <row r="104" hidden="1" spans="1:15">
       <c r="A104" t="s">
         <v>50</v>
       </c>
@@ -20636,7 +20648,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:15">
+    <row r="105" hidden="1" spans="1:15">
       <c r="A105" t="s">
         <v>50</v>
       </c>
@@ -20683,7 +20695,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="106" spans="1:15">
+    <row r="106" hidden="1" spans="1:15">
       <c r="A106" t="s">
         <v>45</v>
       </c>
@@ -20730,7 +20742,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="107" spans="1:15">
+    <row r="107" hidden="1" spans="1:15">
       <c r="A107" t="s">
         <v>48</v>
       </c>
@@ -20777,7 +20789,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="108" spans="1:15">
+    <row r="108" hidden="1" spans="1:15">
       <c r="A108" t="s">
         <v>36</v>
       </c>
@@ -20824,7 +20836,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="109" spans="1:15">
+    <row r="109" hidden="1" spans="1:15">
       <c r="A109" t="s">
         <v>51</v>
       </c>
@@ -20871,7 +20883,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="110" spans="1:15">
+    <row r="110" hidden="1" spans="1:15">
       <c r="A110" t="s">
         <v>47</v>
       </c>
@@ -20918,7 +20930,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="111" spans="1:15">
+    <row r="111" hidden="1" spans="1:15">
       <c r="A111" t="s">
         <v>45</v>
       </c>
@@ -20965,7 +20977,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="112" spans="1:15">
+    <row r="112" hidden="1" spans="1:15">
       <c r="A112" t="s">
         <v>51</v>
       </c>
@@ -21012,7 +21024,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="113" spans="1:15">
+    <row r="113" hidden="1" spans="1:15">
       <c r="A113" t="s">
         <v>54</v>
       </c>
@@ -21059,7 +21071,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="114" spans="1:15">
+    <row r="114" hidden="1" spans="1:15">
       <c r="A114" t="s">
         <v>49</v>
       </c>
@@ -21106,7 +21118,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="115" spans="1:15">
+    <row r="115" hidden="1" spans="1:15">
       <c r="A115" t="s">
         <v>46</v>
       </c>
@@ -21153,7 +21165,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="116" spans="1:15">
+    <row r="116" hidden="1" spans="1:15">
       <c r="A116" t="s">
         <v>55</v>
       </c>
@@ -21200,7 +21212,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="117" spans="1:15">
+    <row r="117" hidden="1" spans="1:15">
       <c r="A117" t="s">
         <v>46</v>
       </c>
@@ -21247,7 +21259,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="118" spans="1:15">
+    <row r="118" hidden="1" spans="1:15">
       <c r="A118" t="s">
         <v>52</v>
       </c>
@@ -21294,7 +21306,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="119" spans="1:15">
+    <row r="119" hidden="1" spans="1:15">
       <c r="A119" t="s">
         <v>54</v>
       </c>
@@ -21341,7 +21353,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="120" spans="1:15">
+    <row r="120" hidden="1" spans="1:15">
       <c r="A120" t="s">
         <v>54</v>
       </c>
@@ -21388,7 +21400,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="121" spans="1:15">
+    <row r="121" hidden="1" spans="1:15">
       <c r="A121" t="s">
         <v>55</v>
       </c>
@@ -21435,7 +21447,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="122" spans="1:15">
+    <row r="122" hidden="1" spans="1:15">
       <c r="A122" t="s">
         <v>48</v>
       </c>
@@ -21482,7 +21494,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="123" spans="1:15">
+    <row r="123" hidden="1" spans="1:15">
       <c r="A123" t="s">
         <v>53</v>
       </c>
@@ -21529,7 +21541,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="124" spans="1:15">
+    <row r="124" hidden="1" spans="1:15">
       <c r="A124" t="s">
         <v>53</v>
       </c>
@@ -21576,7 +21588,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="125" spans="1:15">
+    <row r="125" hidden="1" spans="1:15">
       <c r="A125" t="s">
         <v>36</v>
       </c>
@@ -21623,7 +21635,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="126" spans="1:15">
+    <row r="126" hidden="1" spans="1:15">
       <c r="A126" t="s">
         <v>50</v>
       </c>
@@ -21670,7 +21682,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="127" spans="1:15">
+    <row r="127" hidden="1" spans="1:15">
       <c r="A127" t="s">
         <v>48</v>
       </c>
@@ -21717,7 +21729,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="128" spans="1:15">
+    <row r="128" hidden="1" spans="1:15">
       <c r="A128" t="s">
         <v>53</v>
       </c>
@@ -21764,7 +21776,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="129" spans="1:15">
+    <row r="129" hidden="1" spans="1:15">
       <c r="A129" t="s">
         <v>54</v>
       </c>
@@ -21811,7 +21823,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="130" spans="1:15">
+    <row r="130" hidden="1" spans="1:15">
       <c r="A130" t="s">
         <v>50</v>
       </c>
@@ -21858,7 +21870,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="131" spans="1:15">
+    <row r="131" hidden="1" spans="1:15">
       <c r="A131" t="s">
         <v>53</v>
       </c>
@@ -21905,7 +21917,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="132" spans="1:15">
+    <row r="132" hidden="1" spans="1:15">
       <c r="A132" t="s">
         <v>45</v>
       </c>
@@ -21952,7 +21964,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="133" spans="1:15">
+    <row r="133" hidden="1" spans="1:15">
       <c r="A133" t="s">
         <v>47</v>
       </c>
@@ -21999,7 +22011,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="134" spans="1:15">
+    <row r="134" hidden="1" spans="1:15">
       <c r="A134" t="s">
         <v>48</v>
       </c>
@@ -22046,7 +22058,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="135" spans="1:15">
+    <row r="135" hidden="1" spans="1:15">
       <c r="A135" t="s">
         <v>49</v>
       </c>
@@ -22093,7 +22105,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="136" spans="1:15">
+    <row r="136" hidden="1" spans="1:15">
       <c r="A136" t="s">
         <v>47</v>
       </c>
@@ -22140,7 +22152,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="137" spans="1:15">
+    <row r="137" hidden="1" spans="1:15">
       <c r="A137" t="s">
         <v>54</v>
       </c>
@@ -22187,7 +22199,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="138" spans="1:15">
+    <row r="138" hidden="1" spans="1:15">
       <c r="A138" t="s">
         <v>51</v>
       </c>
@@ -22234,7 +22246,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="139" spans="1:15">
+    <row r="139" hidden="1" spans="1:15">
       <c r="A139" t="s">
         <v>45</v>
       </c>
@@ -22281,7 +22293,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="140" spans="1:15">
+    <row r="140" hidden="1" spans="1:15">
       <c r="A140" t="s">
         <v>36</v>
       </c>
@@ -22328,7 +22340,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="141" spans="1:15">
+    <row r="141" hidden="1" spans="1:15">
       <c r="A141" t="s">
         <v>55</v>
       </c>
@@ -22375,7 +22387,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="142" spans="1:15">
+    <row r="142" hidden="1" spans="1:15">
       <c r="A142" t="s">
         <v>48</v>
       </c>
@@ -22422,7 +22434,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="143" spans="1:15">
+    <row r="143" hidden="1" spans="1:15">
       <c r="A143" t="s">
         <v>45</v>
       </c>
@@ -22469,7 +22481,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="144" spans="1:15">
+    <row r="144" hidden="1" spans="1:15">
       <c r="A144" t="s">
         <v>48</v>
       </c>
@@ -22516,7 +22528,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="145" spans="1:15">
+    <row r="145" hidden="1" spans="1:15">
       <c r="A145" t="s">
         <v>46</v>
       </c>
@@ -22563,7 +22575,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="146" spans="1:15">
+    <row r="146" hidden="1" spans="1:15">
       <c r="A146" t="s">
         <v>45</v>
       </c>
@@ -22610,7 +22622,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="147" spans="1:15">
+    <row r="147" hidden="1" spans="1:15">
       <c r="A147" t="s">
         <v>54</v>
       </c>
@@ -22657,7 +22669,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="148" spans="1:15">
+    <row r="148" hidden="1" spans="1:15">
       <c r="A148" t="s">
         <v>50</v>
       </c>
@@ -22704,7 +22716,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="149" spans="1:15">
+    <row r="149" hidden="1" spans="1:15">
       <c r="A149" t="s">
         <v>46</v>
       </c>
@@ -22751,7 +22763,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="150" spans="1:15">
+    <row r="150" hidden="1" spans="1:15">
       <c r="A150" t="s">
         <v>47</v>
       </c>
@@ -22798,7 +22810,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="151" spans="1:15">
+    <row r="151" hidden="1" spans="1:15">
       <c r="A151" t="s">
         <v>53</v>
       </c>
@@ -22845,7 +22857,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="152" spans="1:15">
+    <row r="152" hidden="1" spans="1:15">
       <c r="A152" t="s">
         <v>45</v>
       </c>
@@ -22892,7 +22904,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="153" spans="1:15">
+    <row r="153" hidden="1" spans="1:15">
       <c r="A153" t="s">
         <v>46</v>
       </c>
@@ -22939,7 +22951,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="154" spans="1:15">
+    <row r="154" hidden="1" spans="1:15">
       <c r="A154" t="s">
         <v>50</v>
       </c>
@@ -22986,7 +22998,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="155" spans="1:15">
+    <row r="155" hidden="1" spans="1:15">
       <c r="A155" t="s">
         <v>46</v>
       </c>
@@ -23033,7 +23045,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="156" spans="1:15">
+    <row r="156" hidden="1" spans="1:15">
       <c r="A156" t="s">
         <v>45</v>
       </c>
@@ -23080,7 +23092,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="157" spans="1:15">
+    <row r="157" hidden="1" spans="1:15">
       <c r="A157" t="s">
         <v>54</v>
       </c>
@@ -23127,7 +23139,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="158" spans="1:15">
+    <row r="158" hidden="1" spans="1:15">
       <c r="A158" t="s">
         <v>50</v>
       </c>
@@ -23174,7 +23186,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="159" spans="1:15">
+    <row r="159" hidden="1" spans="1:15">
       <c r="A159" t="s">
         <v>48</v>
       </c>
@@ -23221,7 +23233,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="160" spans="1:15">
+    <row r="160" hidden="1" spans="1:15">
       <c r="A160" t="s">
         <v>47</v>
       </c>
@@ -23268,7 +23280,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="161" spans="1:15">
+    <row r="161" hidden="1" spans="1:15">
       <c r="A161" t="s">
         <v>51</v>
       </c>
@@ -23315,7 +23327,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="162" spans="1:15">
+    <row r="162" hidden="1" spans="1:15">
       <c r="A162" t="s">
         <v>54</v>
       </c>
@@ -23362,7 +23374,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="163" spans="1:15">
+    <row r="163" hidden="1" spans="1:15">
       <c r="A163" t="s">
         <v>47</v>
       </c>
@@ -23409,7 +23421,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="164" spans="1:15">
+    <row r="164" hidden="1" spans="1:15">
       <c r="A164" t="s">
         <v>55</v>
       </c>
@@ -23456,7 +23468,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="165" spans="1:15">
+    <row r="165" hidden="1" spans="1:15">
       <c r="A165" t="s">
         <v>45</v>
       </c>
@@ -23503,7 +23515,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="166" spans="1:15">
+    <row r="166" hidden="1" spans="1:15">
       <c r="A166" t="s">
         <v>53</v>
       </c>
@@ -23550,7 +23562,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="167" spans="1:15">
+    <row r="167" hidden="1" spans="1:15">
       <c r="A167" t="s">
         <v>36</v>
       </c>
@@ -23597,7 +23609,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="168" spans="1:15">
+    <row r="168" hidden="1" spans="1:15">
       <c r="A168" t="s">
         <v>53</v>
       </c>
@@ -23691,7 +23703,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="170" spans="1:15">
+    <row r="170" hidden="1" spans="1:15">
       <c r="A170" t="s">
         <v>36</v>
       </c>
@@ -23738,7 +23750,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="171" spans="1:15">
+    <row r="171" hidden="1" spans="1:15">
       <c r="A171" t="s">
         <v>55</v>
       </c>
@@ -23785,7 +23797,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="172" spans="1:15">
+    <row r="172" hidden="1" spans="1:15">
       <c r="A172" t="s">
         <v>50</v>
       </c>
@@ -23832,7 +23844,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="173" spans="1:15">
+    <row r="173" hidden="1" spans="1:15">
       <c r="A173" t="s">
         <v>54</v>
       </c>
@@ -23879,7 +23891,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="174" spans="1:15">
+    <row r="174" hidden="1" spans="1:15">
       <c r="A174" t="s">
         <v>54</v>
       </c>
@@ -23926,7 +23938,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="175" spans="1:15">
+    <row r="175" hidden="1" spans="1:15">
       <c r="A175" t="s">
         <v>54</v>
       </c>
@@ -23973,7 +23985,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="176" spans="1:15">
+    <row r="176" hidden="1" spans="1:15">
       <c r="A176" t="s">
         <v>55</v>
       </c>
@@ -24020,7 +24032,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="177" spans="1:15">
+    <row r="177" hidden="1" spans="1:15">
       <c r="A177" t="s">
         <v>52</v>
       </c>
@@ -24067,7 +24079,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="178" spans="1:15">
+    <row r="178" hidden="1" spans="1:15">
       <c r="A178" t="s">
         <v>54</v>
       </c>
@@ -24114,7 +24126,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="179" spans="1:15">
+    <row r="179" hidden="1" spans="1:15">
       <c r="A179" t="s">
         <v>55</v>
       </c>
@@ -24161,7 +24173,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="180" spans="1:15">
+    <row r="180" hidden="1" spans="1:15">
       <c r="A180" t="s">
         <v>53</v>
       </c>
@@ -24208,7 +24220,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="181" spans="1:15">
+    <row r="181" hidden="1" spans="1:15">
       <c r="A181" t="s">
         <v>50</v>
       </c>
@@ -24255,7 +24267,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="182" spans="1:15">
+    <row r="182" hidden="1" spans="1:15">
       <c r="A182" t="s">
         <v>52</v>
       </c>
@@ -24302,7 +24314,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="183" spans="1:15">
+    <row r="183" hidden="1" spans="1:15">
       <c r="A183" t="s">
         <v>36</v>
       </c>
@@ -24349,7 +24361,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="184" spans="1:15">
+    <row r="184" hidden="1" spans="1:15">
       <c r="A184" t="s">
         <v>54</v>
       </c>
@@ -24396,7 +24408,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="185" spans="1:15">
+    <row r="185" hidden="1" spans="1:15">
       <c r="A185" t="s">
         <v>46</v>
       </c>
@@ -24443,7 +24455,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="186" spans="1:15">
+    <row r="186" hidden="1" spans="1:15">
       <c r="A186" t="s">
         <v>52</v>
       </c>
@@ -24490,7 +24502,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="187" spans="1:15">
+    <row r="187" hidden="1" spans="1:15">
       <c r="A187" t="s">
         <v>51</v>
       </c>
@@ -24537,7 +24549,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="188" spans="1:15">
+    <row r="188" hidden="1" spans="1:15">
       <c r="A188" t="s">
         <v>53</v>
       </c>
@@ -24584,7 +24596,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="189" spans="1:15">
+    <row r="189" hidden="1" spans="1:15">
       <c r="A189" t="s">
         <v>47</v>
       </c>
@@ -24631,7 +24643,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="190" spans="1:15">
+    <row r="190" hidden="1" spans="1:15">
       <c r="A190" t="s">
         <v>54</v>
       </c>
@@ -24678,7 +24690,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="191" spans="1:15">
+    <row r="191" hidden="1" spans="1:15">
       <c r="A191" t="s">
         <v>54</v>
       </c>
@@ -24725,7 +24737,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="192" spans="1:15">
+    <row r="192" hidden="1" spans="1:15">
       <c r="A192" t="s">
         <v>48</v>
       </c>
@@ -24772,7 +24784,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="193" spans="1:15">
+    <row r="193" hidden="1" spans="1:15">
       <c r="A193" t="s">
         <v>51</v>
       </c>
@@ -24819,7 +24831,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="194" spans="1:15">
+    <row r="194" hidden="1" spans="1:15">
       <c r="A194" t="s">
         <v>49</v>
       </c>
@@ -24866,7 +24878,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="195" spans="1:15">
+    <row r="195" hidden="1" spans="1:15">
       <c r="A195" t="s">
         <v>53</v>
       </c>
@@ -24913,7 +24925,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="196" spans="1:15">
+    <row r="196" hidden="1" spans="1:15">
       <c r="A196" t="s">
         <v>54</v>
       </c>
@@ -25007,7 +25019,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="198" spans="1:15">
+    <row r="198" hidden="1" spans="1:15">
       <c r="A198" t="s">
         <v>47</v>
       </c>
@@ -25054,7 +25066,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="199" spans="1:15">
+    <row r="199" hidden="1" spans="1:15">
       <c r="A199" t="s">
         <v>46</v>
       </c>
@@ -25101,7 +25113,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="200" spans="1:15">
+    <row r="200" hidden="1" spans="1:15">
       <c r="A200" t="s">
         <v>48</v>
       </c>
@@ -25148,7 +25160,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="201" spans="1:15">
+    <row r="201" hidden="1" spans="1:15">
       <c r="A201" t="s">
         <v>47</v>
       </c>
@@ -25195,7 +25207,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="202" spans="1:15">
+    <row r="202" hidden="1" spans="1:15">
       <c r="A202" t="s">
         <v>47</v>
       </c>
@@ -25242,7 +25254,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="203" spans="1:15">
+    <row r="203" hidden="1" spans="1:15">
       <c r="A203" t="s">
         <v>54</v>
       </c>
@@ -25289,7 +25301,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="204" spans="1:15">
+    <row r="204" hidden="1" spans="1:15">
       <c r="A204" t="s">
         <v>48</v>
       </c>
@@ -25336,7 +25348,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="205" spans="1:15">
+    <row r="205" hidden="1" spans="1:15">
       <c r="A205" t="s">
         <v>51</v>
       </c>
@@ -25383,7 +25395,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="206" spans="1:15">
+    <row r="206" hidden="1" spans="1:15">
       <c r="A206" t="s">
         <v>47</v>
       </c>
@@ -25477,7 +25489,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="208" spans="1:15">
+    <row r="208" hidden="1" spans="1:15">
       <c r="A208" t="s">
         <v>45</v>
       </c>
@@ -25524,7 +25536,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="209" spans="1:15">
+    <row r="209" hidden="1" spans="1:15">
       <c r="A209" t="s">
         <v>46</v>
       </c>
@@ -25571,7 +25583,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="210" spans="1:15">
+    <row r="210" hidden="1" spans="1:15">
       <c r="A210" t="s">
         <v>53</v>
       </c>
@@ -25618,7 +25630,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="211" spans="1:15">
+    <row r="211" hidden="1" spans="1:15">
       <c r="A211" t="s">
         <v>49</v>
       </c>
@@ -25665,7 +25677,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="212" spans="1:15">
+    <row r="212" hidden="1" spans="1:15">
       <c r="A212" t="s">
         <v>49</v>
       </c>
@@ -25712,7 +25724,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="213" spans="1:15">
+    <row r="213" hidden="1" spans="1:15">
       <c r="A213" t="s">
         <v>51</v>
       </c>
@@ -25759,7 +25771,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="214" spans="1:15">
+    <row r="214" hidden="1" spans="1:15">
       <c r="A214" t="s">
         <v>51</v>
       </c>
@@ -25806,7 +25818,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="215" spans="1:15">
+    <row r="215" hidden="1" spans="1:15">
       <c r="A215" t="s">
         <v>49</v>
       </c>
@@ -25853,7 +25865,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="216" spans="1:15">
+    <row r="216" hidden="1" spans="1:15">
       <c r="A216" t="s">
         <v>51</v>
       </c>
@@ -25900,7 +25912,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="217" spans="1:15">
+    <row r="217" hidden="1" spans="1:15">
       <c r="A217" t="s">
         <v>48</v>
       </c>
@@ -25947,7 +25959,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="218" spans="1:15">
+    <row r="218" hidden="1" spans="1:15">
       <c r="A218" t="s">
         <v>54</v>
       </c>
@@ -25994,7 +26006,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="219" spans="1:15">
+    <row r="219" hidden="1" spans="1:15">
       <c r="A219" t="s">
         <v>48</v>
       </c>
@@ -26088,7 +26100,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="221" spans="1:15">
+    <row r="221" hidden="1" spans="1:15">
       <c r="A221" t="s">
         <v>52</v>
       </c>
@@ -26135,7 +26147,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="222" spans="1:15">
+    <row r="222" hidden="1" spans="1:15">
       <c r="A222" t="s">
         <v>46</v>
       </c>
@@ -26182,7 +26194,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="223" spans="1:15">
+    <row r="223" hidden="1" spans="1:15">
       <c r="A223" t="s">
         <v>55</v>
       </c>
@@ -26229,7 +26241,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="224" spans="1:15">
+    <row r="224" hidden="1" spans="1:15">
       <c r="A224" t="s">
         <v>48</v>
       </c>
@@ -26276,7 +26288,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="225" spans="1:15">
+    <row r="225" hidden="1" spans="1:15">
       <c r="A225" t="s">
         <v>55</v>
       </c>
@@ -26323,7 +26335,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="226" spans="1:15">
+    <row r="226" hidden="1" spans="1:15">
       <c r="A226" t="s">
         <v>49</v>
       </c>
@@ -26370,7 +26382,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="227" spans="1:15">
+    <row r="227" hidden="1" spans="1:15">
       <c r="A227" t="s">
         <v>50</v>
       </c>
@@ -26417,7 +26429,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="228" spans="1:15">
+    <row r="228" hidden="1" spans="1:15">
       <c r="A228" t="s">
         <v>49</v>
       </c>
@@ -26464,7 +26476,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="229" spans="1:15">
+    <row r="229" hidden="1" spans="1:15">
       <c r="A229" t="s">
         <v>49</v>
       </c>
@@ -26511,7 +26523,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="230" spans="1:15">
+    <row r="230" hidden="1" spans="1:15">
       <c r="A230" t="s">
         <v>52</v>
       </c>
@@ -26558,7 +26570,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="231" spans="1:15">
+    <row r="231" hidden="1" spans="1:15">
       <c r="A231" t="s">
         <v>49</v>
       </c>
@@ -26605,7 +26617,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="232" spans="1:15">
+    <row r="232" hidden="1" spans="1:15">
       <c r="A232" t="s">
         <v>46</v>
       </c>
@@ -26652,7 +26664,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="233" spans="1:15">
+    <row r="233" hidden="1" spans="1:15">
       <c r="A233" t="s">
         <v>45</v>
       </c>
@@ -26699,7 +26711,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="234" spans="1:15">
+    <row r="234" hidden="1" spans="1:15">
       <c r="A234" t="s">
         <v>55</v>
       </c>
@@ -26793,7 +26805,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="236" spans="1:15">
+    <row r="236" hidden="1" spans="1:15">
       <c r="A236" t="s">
         <v>51</v>
       </c>
@@ -26840,7 +26852,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="237" spans="1:15">
+    <row r="237" hidden="1" spans="1:15">
       <c r="A237" t="s">
         <v>52</v>
       </c>
@@ -26887,7 +26899,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="238" spans="1:15">
+    <row r="238" hidden="1" spans="1:15">
       <c r="A238" t="s">
         <v>49</v>
       </c>
@@ -26934,7 +26946,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="239" spans="1:15">
+    <row r="239" hidden="1" spans="1:15">
       <c r="A239" t="s">
         <v>46</v>
       </c>
@@ -26981,7 +26993,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="240" spans="1:15">
+    <row r="240" hidden="1" spans="1:15">
       <c r="A240" t="s">
         <v>47</v>
       </c>
@@ -27028,7 +27040,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="241" spans="1:15">
+    <row r="241" hidden="1" spans="1:15">
       <c r="A241" t="s">
         <v>53</v>
       </c>
@@ -27075,7 +27087,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="242" spans="1:15">
+    <row r="242" hidden="1" spans="1:15">
       <c r="A242" t="s">
         <v>45</v>
       </c>
@@ -27122,7 +27134,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="243" spans="1:15">
+    <row r="243" hidden="1" spans="1:15">
       <c r="A243" t="s">
         <v>54</v>
       </c>
@@ -27169,7 +27181,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="244" spans="1:15">
+    <row r="244" hidden="1" spans="1:15">
       <c r="A244" t="s">
         <v>51</v>
       </c>
@@ -27216,7 +27228,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="245" spans="1:15">
+    <row r="245" hidden="1" spans="1:15">
       <c r="A245" t="s">
         <v>45</v>
       </c>
@@ -27310,7 +27322,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="247" spans="1:15">
+    <row r="247" hidden="1" spans="1:15">
       <c r="A247" t="s">
         <v>36</v>
       </c>
@@ -27357,7 +27369,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="248" spans="1:15">
+    <row r="248" hidden="1" spans="1:15">
       <c r="A248" t="s">
         <v>53</v>
       </c>
@@ -27404,7 +27416,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="249" spans="1:15">
+    <row r="249" hidden="1" spans="1:15">
       <c r="A249" t="s">
         <v>54</v>
       </c>
@@ -27451,7 +27463,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="250" spans="1:15">
+    <row r="250" hidden="1" spans="1:15">
       <c r="A250" t="s">
         <v>50</v>
       </c>
@@ -27498,7 +27510,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="251" spans="1:15">
+    <row r="251" hidden="1" spans="1:15">
       <c r="A251" t="s">
         <v>46</v>
       </c>
@@ -27545,7 +27557,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="252" spans="1:15">
+    <row r="252" hidden="1" spans="1:15">
       <c r="A252" t="s">
         <v>36</v>
       </c>
@@ -27592,7 +27604,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="253" spans="1:15">
+    <row r="253" hidden="1" spans="1:15">
       <c r="A253" t="s">
         <v>49</v>
       </c>
@@ -27639,7 +27651,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="254" spans="1:15">
+    <row r="254" hidden="1" spans="1:15">
       <c r="A254" t="s">
         <v>36</v>
       </c>
@@ -27686,7 +27698,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="255" spans="1:15">
+    <row r="255" hidden="1" spans="1:15">
       <c r="A255" t="s">
         <v>46</v>
       </c>
@@ -27733,7 +27745,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="256" spans="1:15">
+    <row r="256" hidden="1" spans="1:15">
       <c r="A256" t="s">
         <v>36</v>
       </c>
@@ -27780,7 +27792,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="257" spans="1:15">
+    <row r="257" hidden="1" spans="1:15">
       <c r="A257" t="s">
         <v>45</v>
       </c>
@@ -27827,7 +27839,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="258" spans="1:15">
+    <row r="258" hidden="1" spans="1:15">
       <c r="A258" t="s">
         <v>48</v>
       </c>
@@ -27874,7 +27886,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="259" spans="1:15">
+    <row r="259" hidden="1" spans="1:15">
       <c r="A259" t="s">
         <v>53</v>
       </c>
@@ -27921,7 +27933,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="260" spans="1:15">
+    <row r="260" hidden="1" spans="1:15">
       <c r="A260" t="s">
         <v>49</v>
       </c>
@@ -27968,7 +27980,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="261" spans="1:15">
+    <row r="261" hidden="1" spans="1:15">
       <c r="A261" t="s">
         <v>47</v>
       </c>
@@ -28015,7 +28027,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="262" spans="1:15">
+    <row r="262" hidden="1" spans="1:15">
       <c r="A262" t="s">
         <v>55</v>
       </c>
@@ -28062,7 +28074,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="263" spans="1:15">
+    <row r="263" hidden="1" spans="1:15">
       <c r="A263" t="s">
         <v>52</v>
       </c>
@@ -28109,7 +28121,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="264" spans="1:15">
+    <row r="264" hidden="1" spans="1:15">
       <c r="A264" t="s">
         <v>50</v>
       </c>
@@ -28156,7 +28168,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="265" spans="1:15">
+    <row r="265" hidden="1" spans="1:15">
       <c r="A265" t="s">
         <v>45</v>
       </c>
@@ -28203,7 +28215,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="266" spans="1:15">
+    <row r="266" hidden="1" spans="1:15">
       <c r="A266" t="s">
         <v>54</v>
       </c>
@@ -28250,7 +28262,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="267" spans="1:15">
+    <row r="267" hidden="1" spans="1:15">
       <c r="A267" t="s">
         <v>53</v>
       </c>
@@ -28297,7 +28309,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="268" spans="1:15">
+    <row r="268" hidden="1" spans="1:15">
       <c r="A268" t="s">
         <v>45</v>
       </c>
@@ -28344,7 +28356,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="269" spans="1:15">
+    <row r="269" hidden="1" spans="1:15">
       <c r="A269" t="s">
         <v>48</v>
       </c>
@@ -28391,7 +28403,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="270" spans="1:15">
+    <row r="270" hidden="1" spans="1:15">
       <c r="A270" t="s">
         <v>55</v>
       </c>
@@ -28438,7 +28450,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="271" spans="1:15">
+    <row r="271" hidden="1" spans="1:15">
       <c r="A271" t="s">
         <v>52</v>
       </c>
@@ -28485,7 +28497,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="272" spans="1:15">
+    <row r="272" hidden="1" spans="1:15">
       <c r="A272" t="s">
         <v>46</v>
       </c>
@@ -28532,7 +28544,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="273" spans="1:15">
+    <row r="273" hidden="1" spans="1:15">
       <c r="A273" t="s">
         <v>46</v>
       </c>
@@ -28579,7 +28591,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="274" spans="1:15">
+    <row r="274" hidden="1" spans="1:15">
       <c r="A274" t="s">
         <v>54</v>
       </c>
@@ -28626,7 +28638,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="275" spans="1:15">
+    <row r="275" hidden="1" spans="1:15">
       <c r="A275" t="s">
         <v>54</v>
       </c>
@@ -28673,7 +28685,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="276" spans="1:15">
+    <row r="276" hidden="1" spans="1:15">
       <c r="A276" t="s">
         <v>51</v>
       </c>
@@ -28720,7 +28732,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="277" spans="1:15">
+    <row r="277" hidden="1" spans="1:15">
       <c r="A277" t="s">
         <v>50</v>
       </c>
@@ -28767,7 +28779,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="278" spans="1:15">
+    <row r="278" hidden="1" spans="1:15">
       <c r="A278" t="s">
         <v>52</v>
       </c>
@@ -28814,7 +28826,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="279" spans="1:15">
+    <row r="279" hidden="1" spans="1:15">
       <c r="A279" t="s">
         <v>52</v>
       </c>
@@ -28861,7 +28873,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="280" spans="1:15">
+    <row r="280" hidden="1" spans="1:15">
       <c r="A280" t="s">
         <v>46</v>
       </c>
@@ -28908,7 +28920,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="281" spans="1:15">
+    <row r="281" hidden="1" spans="1:15">
       <c r="A281" t="s">
         <v>46</v>
       </c>
@@ -28955,7 +28967,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="282" spans="1:15">
+    <row r="282" hidden="1" spans="1:15">
       <c r="A282" t="s">
         <v>55</v>
       </c>
@@ -29002,7 +29014,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="283" spans="1:15">
+    <row r="283" hidden="1" spans="1:15">
       <c r="A283" t="s">
         <v>48</v>
       </c>
@@ -29049,7 +29061,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="284" spans="1:15">
+    <row r="284" hidden="1" spans="1:15">
       <c r="A284" t="s">
         <v>47</v>
       </c>
@@ -29096,7 +29108,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="285" spans="1:15">
+    <row r="285" hidden="1" spans="1:15">
       <c r="A285" t="s">
         <v>47</v>
       </c>
@@ -29143,7 +29155,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="286" spans="1:15">
+    <row r="286" hidden="1" spans="1:15">
       <c r="A286" t="s">
         <v>46</v>
       </c>
@@ -29190,7 +29202,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="287" spans="1:15">
+    <row r="287" hidden="1" spans="1:15">
       <c r="A287" t="s">
         <v>52</v>
       </c>
@@ -29237,7 +29249,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="288" spans="1:15">
+    <row r="288" hidden="1" spans="1:15">
       <c r="A288" t="s">
         <v>50</v>
       </c>
@@ -29284,7 +29296,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="289" spans="1:15">
+    <row r="289" hidden="1" spans="1:15">
       <c r="A289" t="s">
         <v>48</v>
       </c>
@@ -29331,7 +29343,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="290" spans="1:15">
+    <row r="290" hidden="1" spans="1:15">
       <c r="A290" t="s">
         <v>48</v>
       </c>
@@ -29378,7 +29390,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="291" spans="1:15">
+    <row r="291" hidden="1" spans="1:15">
       <c r="A291" t="s">
         <v>50</v>
       </c>
@@ -29425,7 +29437,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="292" spans="1:15">
+    <row r="292" hidden="1" spans="1:15">
       <c r="A292" t="s">
         <v>49</v>
       </c>
@@ -29472,7 +29484,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="293" spans="1:15">
+    <row r="293" hidden="1" spans="1:15">
       <c r="A293" t="s">
         <v>51</v>
       </c>
@@ -29519,7 +29531,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="294" spans="1:15">
+    <row r="294" hidden="1" spans="1:15">
       <c r="A294" t="s">
         <v>51</v>
       </c>
@@ -29566,7 +29578,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="295" spans="1:15">
+    <row r="295" hidden="1" spans="1:15">
       <c r="A295" t="s">
         <v>53</v>
       </c>
@@ -29613,7 +29625,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="296" spans="1:15">
+    <row r="296" hidden="1" spans="1:15">
       <c r="A296" t="s">
         <v>55</v>
       </c>
@@ -29660,7 +29672,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="297" spans="1:15">
+    <row r="297" hidden="1" spans="1:15">
       <c r="A297" t="s">
         <v>49</v>
       </c>
@@ -29707,7 +29719,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="298" spans="1:15">
+    <row r="298" hidden="1" spans="1:15">
       <c r="A298" t="s">
         <v>36</v>
       </c>
@@ -29754,7 +29766,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="299" spans="1:15">
+    <row r="299" hidden="1" spans="1:15">
       <c r="A299" t="s">
         <v>46</v>
       </c>
@@ -29801,7 +29813,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="300" spans="1:15">
+    <row r="300" hidden="1" spans="1:15">
       <c r="A300" t="s">
         <v>53</v>
       </c>
@@ -29848,7 +29860,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="301" spans="1:15">
+    <row r="301" hidden="1" spans="1:15">
       <c r="A301" t="s">
         <v>53</v>
       </c>
@@ -32711,7 +32723,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1982d45a-6c1e-4de4-828e-4177c265aab3}</x14:id>
+          <x14:id>{78daf04d-f636-4c42-8bc3-69d53ca9ce67}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -32725,7 +32737,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1982d45a-6c1e-4de4-828e-4177c265aab3}">
+          <x14:cfRule type="dataBar" id="{78daf04d-f636-4c42-8bc3-69d53ca9ce67}">
             <x14:dataBar minLength="10" maxLength="90" negativeBarColorSameAsPositive="1">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>